<commit_message>
Prep checklist: assign COSEM LO/MC tasks, Gerry, Fujimoto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レイアウト" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'準備一覧'!$A$4:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'準備一覧'!$A$4:$L$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'準備一覧'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -760,7 +760,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>池田</t>
+          <t>Gerry</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>RT のコメント用紙（各席）、アジェンダ。部数は配席の席数＋予備。</t>
+          <t>RT のコメント用紙、アジェンダ。テーブルに置く。部数は配席の席数＋予備。</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>受付で配るか各席に置くかを決める。</t>
+          <t>テーブルに置く。部数は席数を目安に決める。</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>【TBC】</t>
+          <t>藤本</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1031,32 +1031,32 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>〜10/27</t>
+          <t>〜10/24</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>資料</t>
+          <t>依頼</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>発音付きの登壇者・発言者名簿を MC へ</t>
+          <t>COSEM（LO・MC）への設営依頼</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>氏名・肩書・発音。RT と TS の最終順。</t>
+          <t>配布物のテーブル配置、国名プレート・席札の配置、マイクの音出し確認を 28 日朝に LO・MC に頼む。この一覧の該当行と配席図を Sylvia に送る。</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>吉田</t>
+          <t>荒木田</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>荒木田、池田</t>
+          <t>児玉</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -1064,145 +1064,153 @@
           <t>―</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
       <c r="K14" s="6" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr">
         <is>
+          <t>10/8 ブリーフィングで LO・MC の支援を Sylvia が申出</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>出発前</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>〜10/27</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>資料</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>発音付きの登壇者・発言者名簿を MC へ</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>氏名・肩書・発音。RT と TS の最終順。</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>吉田</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>荒木田、池田</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
           <t>10/27 送付</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>10/27（火）会場下見（Peridot は使えない）</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-      <c r="L15" s="5" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+      <c r="L16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>10/27</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>09:00-11:00</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>確認</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>全員で会場下見・動線確認</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Hall 3、Peridot、Tourmaline 207、ランチ会場、バス乗り場、Hotel Mi・Dorsett からの徒歩経路。</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>児玉</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>全員</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>全体</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr"/>
-      <c r="K16" s="6" t="inlineStr"/>
-      <c r="L16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>10/28（水）Day 1 朝</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>10/28</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>08:00-08:15</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>確認</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>入室・業者設営の確認</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓・電源が配席図どおりか。違いがあれば Sylvia と業者に伝える。</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>荒木田</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>児玉</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>全体</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr"/>
-      <c r="K18" s="6" t="inlineStr"/>
-      <c r="L18" s="7" t="inlineStr"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
+      <c r="L18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
@@ -1215,44 +1223,40 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>08:00-08:45</t>
+          <t>08:00-08:15</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>設営</t>
+          <t>確認</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>バナー（A 型フレーム）の組立・設置</t>
+          <t>入室・業者設営の確認</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>位置は Sylvia と確認した場所。マジックテープで固定。</t>
+          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓・電源が配席図どおりか。違いがあれば Sylvia と業者に伝える。</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>池田</t>
+          <t>荒木田</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Gerry</t>
+          <t>児玉</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr"/>
       <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="7" t="inlineStr"/>
     </row>
@@ -1267,7 +1271,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>08:00-09:00</t>
+          <t>08:00-08:45</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1277,30 +1281,34 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>事務局部屋（Tourmaline 207）の立上げ</t>
+          <t>バナー（A 型フレーム）の組立・設置</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>荷物・配布物の保管、ポータブルプリンター、延長コード。</t>
+          <t>位置は Sylvia と確認した場所。マジックテープで固定。</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
+          <t>池田</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
           <t>Gerry</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>児玉</t>
-        </is>
-      </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
       <c r="K20" s="6" t="inlineStr"/>
       <c r="L20" s="7" t="inlineStr"/>
     </row>
@@ -1315,37 +1323,37 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>08:15-09:00</t>
+          <t>08:00-09:00</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>機材</t>
+          <t>設営</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>AV 卓に PC 3 台を接続</t>
+          <t>事務局部屋（Tourmaline 207）の立上げ</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Zoom 用（藤本）、進行スライド用（池田）、発表用（Gerry）。HDMI 2 系統をスイッチャーへ、電源、切替を AV オペと確認。</t>
+          <t>荷物・配布物の保管、ポータブルプリンター、延長コード。</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>池田</t>
+          <t>Gerry</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>藤本、Gerry</t>
+          <t>児玉</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>J</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr"/>
@@ -1373,36 +1381,32 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>カメラの設置・画角確認</t>
+          <t>AV 卓に PC 3 台を接続</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>後方中央。演台・U 字・前方卓が入るか。映像を AV 卓の Zoom 用 PC へ。業者カメラの場合は業者オペと確認し、ADRC のカメラは予備。</t>
+          <t>Zoom 用（藤本）、進行スライド用（池田）、発表用（Gerry）。HDMI 2 系統をスイッチャーへ、電源、切替を AV オペと確認。</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>荒木田</t>
+          <t>池田</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>塩見</t>
+          <t>藤本、Gerry</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr"/>
       <c r="K22" s="6" t="inlineStr"/>
-      <c r="L22" s="7" t="inlineStr">
-        <is>
-          <t>業者カメラか ADRC カメラか【TBC】</t>
-        </is>
-      </c>
+      <c r="L22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
@@ -1415,7 +1419,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>08:30-09:15</t>
+          <t>08:15-09:00</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1425,12 +1429,12 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>マイクの音出し</t>
+          <t>カメラの設置・画角確認</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>U 字（2 席に 1 本）、前方卓、教室型の 2 本、スタンド 4、ハンド 2、演台。席に座って一本ずつ確認。</t>
+          <t>後方中央。演台・U 字・前方卓が入るか。映像を AV 卓の Zoom 用 PC へ。業者カメラの場合は業者オペと確認し、ADRC のカメラは予備。</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1440,21 +1444,21 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>吉田、AV オペ</t>
+          <t>塩見</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>A・B・D</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr"/>
       <c r="K23" s="6" t="inlineStr"/>
-      <c r="L23" s="7" t="inlineStr"/>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>業者カメラか ADRC カメラか【TBC】</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
@@ -1467,42 +1471,50 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>08:30-09:30</t>
+          <t>08:30-09:15</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>機材</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Zoom Webinar 接続テスト</t>
+          <t>マイクの音出し</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>神戸がホスト（日本時間 09:30〜）。会場音声→Zoom、Zoom の音声→会場スピーカー、カメラ映像、スライド共有、録画、Q&amp;A。</t>
+          <t>U 字（2 席に 1 本）、前方卓、教室型の 2 本、スタンド 4、ハンド 2、演台。席に座って一本ずつ確認。</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>藤本</t>
+          <t>COSEM（LO・MC）</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>中村、山口（神戸）、荒木田</t>
+          <t>荒木田（立会）、AV オペ</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr"/>
+          <t>A・B・D</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
       <c r="K24" s="6" t="inlineStr"/>
-      <c r="L24" s="7" t="inlineStr"/>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>COSEM に依頼</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
@@ -1525,12 +1537,12 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Sentio のテスト</t>
+          <t>Zoom Webinar 接続テスト</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>神戸が共有を開始→QR を受信→読み取りと言語選択を確認。テストの共有は必ず終了する（6 時間で失効、本番は 12:40 開始）。</t>
+          <t>神戸がホスト（日本時間 09:30〜）。会場音声→Zoom、Zoom の音声→会場スピーカー、カメラ映像、スライド共有、録画、Q&amp;A。</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -1540,7 +1552,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>中村（神戸）</t>
+          <t>中村、山口（神戸）、荒木田</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
@@ -1568,27 +1580,27 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>スライド</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>進行スライドの確認</t>
+          <t>Sentio のテスト</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Day1 の PPT 01〜12、国名スライドの順と表示・非表示、待機画面を投影。</t>
+          <t>神戸が共有を開始→QR を受信→読み取りと言語選択を確認。テストの共有は必ず終了する（6 時間で失効、本番は 12:40 開始）。</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>池田</t>
+          <t>藤本</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>荒木田</t>
+          <t>中村（神戸）</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
@@ -1611,44 +1623,40 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>09:00-10:00</t>
+          <t>08:30-09:30</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>名札</t>
+          <t>スライド</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>国名プレート・席札の配置</t>
+          <t>進行スライドの確認</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>U 字 28、側面列、教室型の指定席、前方のモデレーター卓。配席図どおり。</t>
+          <t>Day1 の PPT 01〜12、国名スライドの順と表示・非表示、待機画面を投影。</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>吉田</t>
+          <t>池田</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>LO</t>
+          <t>荒木田</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>A・B・C・D</t>
-        </is>
-      </c>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr"/>
       <c r="K27" s="6" t="inlineStr"/>
       <c r="L27" s="7" t="inlineStr"/>
     </row>
@@ -1668,32 +1676,32 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>配布物</t>
+          <t>名札</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>各席の配布物セット</t>
+          <t>国名プレート・席札の配置</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>コメント用紙、アジェンダ、ペン。Annual Report は受付か各席か（藤本の判断）。</t>
+          <t>U 字 28、側面列、教室型の指定席、前方のモデレーター卓。配席図どおり。</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>塩見</t>
+          <t>COSEM（LO・MC）</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>藤本、LO</t>
+          <t>吉田（配席図で指示・確認）</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>A・C・D</t>
+          <t>A・B・C・D</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -1702,7 +1710,11 @@
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr"/>
-      <c r="L28" s="7" t="inlineStr"/>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>COSEM に依頼</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -1715,44 +1727,48 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>09:15-10:00</t>
+          <t>09:00-10:00</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>受付</t>
+          <t>配布物</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>受付デスクの設営（Peridot 前）</t>
+          <t>テーブルへの配布物セット</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>名簿、名札の予備・ストラップ、一般参加者向け案内（パスは Hall 3 で各自印刷）。</t>
+          <t>コメント用紙、アジェンダ、ペン、Annual Report をテーブルに置く。</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>藤中</t>
+          <t>COSEM（LO・MC）</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>田中</t>
+          <t>塩見（指示・確認）、藤本</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="inlineStr"/>
+          <t>A・C・D</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
       <c r="K29" s="6" t="inlineStr"/>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>藤中・田中は 09:00 まで Dorsett</t>
+          <t>COSEM に依頼</t>
         </is>
       </c>
     </row>
@@ -1767,42 +1783,46 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>09:15-10:00</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>受付</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>ベル・タイマーの確認</t>
+          <t>受付デスクの設営（Peridot 前）</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>2023 方式のベル。1 分前 1 回、30 秒前 2 回、終了 3 回。</t>
+          <t>名簿、名札の予備・ストラップ、一般参加者向け案内（パスは Hall 3 で各自印刷）。</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>吉田</t>
+          <t>藤中</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Gerry</t>
+          <t>田中</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>H</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr"/>
       <c r="K30" s="6" t="inlineStr"/>
-      <c r="L30" s="7" t="inlineStr"/>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>藤中・田中は 09:00 まで Dorsett</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -1815,42 +1835,42 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>10:00-10:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>―</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Joint Opening（Hall 3）</t>
+          <t>ベル・タイマーの確認</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>随行の職員は Hall 3。残りの職員は設営を続ける。</t>
+          <t>2023 方式のベル。1 分前 1 回、30 秒前 2 回、終了 3 回。</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>宮木、児玉</t>
-        </is>
-      </c>
-      <c r="H31" s="7" t="inlineStr"/>
+          <t>吉田</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Gerry</t>
+        </is>
+      </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>―</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr"/>
       <c r="K31" s="6" t="inlineStr"/>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>随行者は動態表で確定</t>
-        </is>
-      </c>
+      <c r="L31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -1863,46 +1883,42 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>10:30-11:30</t>
+          <t>10:00-10:30</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>確認</t>
+          <t>―</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>MC との台本・立ち位置の確認</t>
+          <t>Joint Opening（Hall 3）</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>12:40 アナウンス、Opening（演台）、集合写真、RT（モデレーター卓）。発音の確認。</t>
+          <t>随行の職員は Hall 3。残りの職員は設営を続ける。</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>荒木田</t>
-        </is>
-      </c>
-      <c r="H32" s="7" t="inlineStr">
-        <is>
-          <t>吉田、池田、MC 2 名</t>
-        </is>
-      </c>
+          <t>宮木、児玉</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr"/>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J32" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr"/>
       <c r="K32" s="6" t="inlineStr"/>
-      <c r="L32" s="7" t="inlineStr"/>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t>随行者は動態表で確定</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -1925,22 +1941,22 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>演台の移動と集合写真の段取り</t>
+          <t>MC との台本・立ち位置の確認</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Opening はステージ中央、終了後にそで（AV 卓側）へ移す担当。集合写真のステージ上の並びと誘導順（U 字から）。撮影位置。</t>
+          <t>12:40 アナウンス、Opening（演台）、集合写真、RT（モデレーター卓）。発音の確認。</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>池田</t>
+          <t>荒木田</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>吉田、田中、藤本（撮影）、LO</t>
+          <t>吉田、池田、MC 2 名</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
@@ -1954,11 +1970,7 @@
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr"/>
-      <c r="L33" s="7" t="inlineStr">
-        <is>
-          <t>対象範囲は ADRC で決定【TBC】</t>
-        </is>
-      </c>
+      <c r="L33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -1971,38 +1983,50 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>11:45-12:30</t>
+          <t>10:30-11:30</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>―</t>
+          <t>確認</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>交代で昼食</t>
+          <t>演台の移動と集合写真の段取り</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>AV 卓と受付は常に 1 名残す。</t>
+          <t>Opening はステージ中央、終了後にそで（AV 卓側）へ移す担当。集合写真のステージ上の並びと誘導順（U 字から）。撮影位置。</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>各自</t>
-        </is>
-      </c>
-      <c r="H34" s="7" t="inlineStr"/>
+          <t>池田</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>吉田、田中、藤本（撮影）、LO</t>
+        </is>
+      </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>―</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="inlineStr"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
       <c r="K34" s="6" t="inlineStr"/>
-      <c r="L34" s="7" t="inlineStr"/>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>対象範囲は ADRC で決定【TBC】</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
@@ -2015,7 +2039,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>11:45-12:30</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2025,27 +2049,23 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>全員配置</t>
+          <t>交代で昼食</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>受付（藤中・田中）、AV 卓（池田・藤本・荒木田）、RT（吉田・Gerry）、記録（塩見）。</t>
+          <t>AV 卓と受付は常に 1 名残す。</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>荒木田</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>全員</t>
-        </is>
-      </c>
+          <t>各自</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr"/>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>全体</t>
+          <t>―</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr"/>
@@ -2063,37 +2083,37 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>―</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Webinar 開始・録画、Sentio 本番共有開始</t>
+          <t>全員配置</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>神戸が開始。届いた QR を情報スライドに貼る（藤本）。卓上の案内カードを印刷して配る（田中）。</t>
+          <t>受付（藤中・田中）、AV 卓（池田・藤本・荒木田）、RT（吉田・Gerry）、記録（塩見）。</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>藤本</t>
+          <t>荒木田</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>中村（神戸）、田中</t>
+          <t>全員</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>F・H</t>
+          <t>全体</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr"/>
@@ -2111,37 +2131,37 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>15:00-15:15</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>転換</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>SC への転換</t>
+          <t>Webinar 開始・録画、Sentio 本番共有開始</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>RT 資料の回収（吉田・塩見）、前方席の名札を SC 用に差替（吉田・田中）、SC 用 Zoom（別リンク）の接続。</t>
+          <t>神戸が開始。届いた QR を情報スライドに貼る（藤本）。卓上の案内カードを印刷して配る（田中）。</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>吉田</t>
+          <t>藤本</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>塩見、田中、池田（Zoom）</t>
+          <t>中村（神戸）、田中</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>A・B・F</t>
+          <t>F・H</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr"/>
@@ -2159,33 +2179,37 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>16:15-16:30</t>
+          <t>15:00-15:15</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>片付け</t>
+          <t>転換</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>機材の保管</t>
+          <t>SC への転換</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>PC・カメラは事務局部屋へ。家具・国名プレートは翌日のまま。</t>
+          <t>RT 資料の回収（吉田・塩見）、前方席の名札を SC 用に差替（吉田・田中）、SC 用 Zoom（別リンク）の接続。</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>各持参者</t>
-        </is>
-      </c>
-      <c r="H38" s="7" t="inlineStr"/>
+          <t>吉田</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>塩見、田中、池田（Zoom）</t>
+        </is>
+      </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
-          <t>F・J</t>
+          <t>A・B・F</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr"/>
@@ -2193,74 +2217,66 @@
       <c r="L38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="A39" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>16:15-16:30</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>片付け</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>機材の保管</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>PC・カメラは事務局部屋へ。家具・国名プレートは翌日のまま。</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>各持参者</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>F・J</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr"/>
+      <c r="K39" s="6" t="inlineStr"/>
+      <c r="L39" s="7" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>10/29（木）Day 2 朝</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n"/>
-      <c r="C39" s="5" t="n"/>
-      <c r="D39" s="5" t="n"/>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="5" t="n"/>
-      <c r="L39" s="5" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>10/29</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>08:00-08:30</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>名札</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>前方卓の席札を差替</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>TS 登壇者・モデレーター・Co-Chair。RT Part 2 の国名プレートは U 字に残す。</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>池田</t>
-        </is>
-      </c>
-      <c r="H40" s="7" t="inlineStr">
-        <is>
-          <t>吉田</t>
-        </is>
-      </c>
-      <c r="I40" s="7" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J40" s="8" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="inlineStr"/>
-      <c r="L40" s="7" t="inlineStr"/>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
+      <c r="K40" s="5" t="n"/>
+      <c r="L40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
@@ -2273,40 +2289,44 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>08:00-08:45</t>
+          <t>08:00-08:30</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>機材</t>
+          <t>名札</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>PC・カメラ・マイクの再接続</t>
+          <t>前方卓の席札を差替</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>前日と同じ確認を短く。</t>
+          <t>TS 登壇者・モデレーター・Co-Chair。RT Part 2 の国名プレートは U 字に残す。</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>荒木田</t>
+          <t>池田</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>藤本、池田</t>
+          <t>吉田</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>F・I</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="inlineStr"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
       <c r="K41" s="6" t="inlineStr"/>
       <c r="L41" s="7" t="inlineStr"/>
     </row>
@@ -2321,37 +2341,37 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>08:15-08:45</t>
+          <t>08:00-08:45</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>機材</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>Zoom 接続テスト</t>
+          <t>PC・カメラ・マイクの再接続</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>神戸（日本時間 09:15〜）。</t>
+          <t>前日と同じ確認を短く。</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>藤本</t>
+          <t>荒木田</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>中村（神戸）</t>
+          <t>藤本、池田</t>
         </is>
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>F・I</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr"/>
@@ -2369,32 +2389,32 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>08:00-08:45</t>
+          <t>08:15-08:45</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>スライド</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>TS 発表スライドを発表用 PC に集約</t>
+          <t>Zoom 接続テスト</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>ファイル名「順番_組織」。クリッカーと予備電池。</t>
+          <t>神戸（日本時間 09:15〜）。</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Gerry</t>
+          <t>藤本</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>池田</t>
+          <t>中村（神戸）</t>
         </is>
       </c>
       <c r="I43" s="7" t="inlineStr">
@@ -2417,37 +2437,37 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>08:30-08:50</t>
+          <t>08:00-08:45</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>スライド</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>登壇者集合・発表確認</t>
+          <t>TS 発表スライドを発表用 PC に集約</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>順番、持ち時間、演台、質疑の進め方。</t>
+          <t>ファイル名「順番_組織」。クリッカーと予備電池。</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
+          <t>Gerry</t>
+        </is>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
           <t>池田</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
-        <is>
-          <t>Mizan</t>
-        </is>
-      </c>
       <c r="I44" s="7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr"/>
@@ -2465,37 +2485,37 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>08:00-09:00</t>
+          <t>08:30-08:50</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>誘導</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>ホテル→EXPO の誘導</t>
+          <t>登壇者集合・発表確認</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Dorsett（田中・塩見）、Hotel Mi（吉田）。</t>
+          <t>順番、持ち時間、演台、質疑の進め方。</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>田中</t>
+          <t>池田</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>塩見、吉田</t>
+          <t>Mizan</t>
         </is>
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>―</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr"/>
@@ -2513,37 +2533,37 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>08:55</t>
+          <t>08:00-09:00</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>配信</t>
+          <t>誘導</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Sentio 本番共有開始</t>
+          <t>ホテル→EXPO の誘導</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>QR をスライドに貼る（28 日の QR は失効）。卓上カードを印刷して配る。</t>
+          <t>Dorsett（田中・塩見）、Hotel Mi（吉田）。</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>藤本</t>
+          <t>田中</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>中村（神戸）、田中</t>
+          <t>塩見、吉田</t>
         </is>
       </c>
       <c r="I46" s="7" t="inlineStr">
         <is>
-          <t>F・H</t>
+          <t>―</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr"/>
@@ -2561,37 +2581,37 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>11:30-11:45</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>転換</t>
+          <t>配信</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>閉会への転換</t>
+          <t>Sentio 本番共有開始</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Summary スライドの差込（Gerry→池田）。前方の登壇者席札を撤去、三浦センター長の席札。</t>
+          <t>QR をスライドに貼る（28 日の QR は失効）。卓上カードを印刷して配る。</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>池田</t>
+          <t>藤本</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>Gerry、吉田</t>
+          <t>中村（神戸）、田中</t>
         </is>
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>B・F</t>
+          <t>F・H</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr"/>
@@ -2609,51 +2629,99 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>12:00-12:30</t>
+          <t>11:30-11:45</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>片付け</t>
+          <t>転換</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>撤収</t>
+          <t>閉会への転換</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>機材回収、配布物の残り、事務局部屋。フィールドトリップ引率者は 12:50 にバス乗り場。</t>
+          <t>Summary スライドの差込（Gerry→池田）。前方の登壇者席札を撤去、三浦センター長の席札。</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>児玉</t>
+          <t>池田</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>藤中、各持参者</t>
+          <t>Gerry、吉田</t>
         </is>
       </c>
       <c r="I48" s="7" t="inlineStr">
         <is>
-          <t>全体</t>
+          <t>B・F</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr"/>
       <c r="K48" s="6" t="inlineStr"/>
       <c r="L48" s="7" t="inlineStr"/>
     </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>10/29</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>12:00-12:30</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>片付け</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>撤収</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>機材回収、配布物の残り、事務局部屋。フィールドトリップ引率者は 12:50 にバス乗り場。</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>児玉</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>藤中、各持参者</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr"/>
+      <c r="L49" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L48"/>
+  <autoFilter ref="A4:L49"/>
   <mergeCells count="5">
     <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A16:L16"/>
     <mergeCell ref="A5:L5"/>
-    <mergeCell ref="A17:L17"/>
-    <mergeCell ref="A39:L39"/>
+    <mergeCell ref="A40:L40"/>
+    <mergeCell ref="A18:L18"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Prep checklist layout sheet from EXPO floor plan 8 Oct
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,12 +58,6 @@
       <name val="Meiryo UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -116,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -137,7 +131,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -218,6 +211,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9525000" cy="10086975"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1238,7 +1261,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓・電源が配席図どおりか。違いがあれば Sylvia と業者に伝える。</t>
+          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓が EXPO 図面（8 Oct）どおりか。電源: AV 卓・事務局・カメラ位置は既存コンセント＋延長コード、側面列と教室型は見積の結果どおりか。違いがあれば Sylvia と業者に伝える。</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2734,217 +2757,210 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Peridot レイアウト（配席図をここに貼る）</t>
+          <t>Peridot レイアウト（EXPO 図面 8 Oct に電源の要否を記入）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>最新の配席図（児玉さん 修正案1005〈インドネシア参加時〉、または EXPO の V4 図面）を A4 から貼り付ける。準備一覧の「場所」の記号は下の凡例に対応。</t>
+          <t>図は EXPO の ACDR Workshop Floorplan（8 Oct）の Peridot 部分。赤い PP は既存コンセント。A〜C の色枠は電源の扱い（右の凡例）。国名プレートの席割りは配席表（児玉さん 修正案1005）による。準備一覧の「場所」の記号は下の凡例に対応。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>（配席図の貼付位置: A4〜L28）</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
           <t>記号</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>場所</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>U 字（28 席）</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>メンバー国の団長、アドバイザー国、Singapore、ADRC。卓上マイク 2 席に 1 本</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>ステージ・前方卓・演台</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>左卓＝モデレーター（Day2 は Co-Chair も）、右卓＝TS 登壇者。演台は Opening・Closing は中央、それ以外はそで</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>側面列（左・右）</t>
-        </is>
-      </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>2 人目の代表、パートナー機関、事務方</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>側面列（左 12・右 12）</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>2 人目の代表、パートナー機関、事務方。電源: 左は左壁から延長タップ、右は追加（見積次第）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>教室型（30 席）</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>リソース（内閣府、仙台市、JAXA、BRIN、Google ほか）。1 列目に卓上マイク 2 本</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>教室型（30 席、5 卓×3 列）</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>リソース（内閣府、仙台市、JAXA、BRIN、Google ほか）。1 列目に卓上マイク 2 本。電源は追加（見積次第）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>シアター席（後方）</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>シアター席（後方 54 席）</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>一般参加者ほか自由席</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>AV 卓</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>PC 3 台（Zoom 用・進行スライド用・発表用）、スイッチャー</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>AV 卓（前方左）</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>PC 3 台（Zoom 用・進行スライド用・発表用）、スイッチャー。脇の既存コンセント</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
-        <is>
-          <t>事務局ブロック（8 席）</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>AV 卓の隣。ADRC 職員</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>ADRC 事務局（AV 卓の隣、前方左 2 卓）</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>ADRC 職員。脇の既存コンセント</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>受付（Peridot 前）</t>
         </is>
       </c>
-      <c r="C38" s="12" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>藤中・田中</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>カメラ位置（後方中央）</t>
         </is>
       </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>三脚、HDMI 10m で AV 卓へ</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>三脚、HDMI で AV 卓へ（前方左まで約 20m 以上、延長が必要か業者と確認）。後方壁の既存コンセント</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>事務局部屋（Tourmaline 207）</t>
         </is>
       </c>
-      <c r="C40" s="12" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>荷物・配布物・プリンター</t>
         </is>
@@ -2952,5 +2968,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Power plan and layout for Peridot 204-206; theatre 40 seat issue
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
@@ -222,7 +222,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9525000" cy="10086975"/>
+    <ext cx="9525000" cy="10296525"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -825,7 +825,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>U 字 28、側面列、教室型の指定席、前方卓（Day1 モデレーター／Day2 TS 登壇者・Co-Chair／SC 用／閉会用）。COSEM が作る参加者名札（パス）とは別。</t>
+          <t>U 字 30、側面列、教室型の指定席、前方卓（Day1 モデレーター／Day2 TS 登壇者・Co-Chair／SC 用／閉会用）。COSEM が作る参加者名札（パス）とは別。</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓が EXPO 図面（8 Oct）どおりか。電源: AV 卓・事務局・カメラ位置は既存コンセント＋延長コード、側面列と教室型は見積の結果どおりか。違いがあれば Sylvia と業者に伝える。</t>
+          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓が EXPO 図面（Peridot 204-206）どおりか。電源: AV 卓・事務局・カメラ位置は既存コンセント＋延長コード、側面列と教室型は見積の結果どおりか。違いがあれば Sylvia と業者に伝える。</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>U 字 28、側面列、教室型の指定席、前方のモデレーター卓。配席図どおり。</t>
+          <t>U 字 30、側面列、教室型の指定席、前方のモデレーター卓。配席図どおり。</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -2768,14 +2768,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Peridot レイアウト（EXPO 図面 8 Oct に電源の要否を記入）</t>
+          <t>Peridot 204-206 レイアウト（EXPO 図面に電源の要否を記入）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>図は EXPO の ACDR Workshop Floorplan（8 Oct）の Peridot 部分。赤い PP は既存コンセント。A〜C の色枠は電源の扱い（右の凡例）。国名プレートの席割りは配席表（児玉さん 修正案1005）による。準備一覧の「場所」の記号は下の凡例に対応。</t>
+          <t>図は EXPO の ACDR Workshop Floorplan（Peridot 204-206、10/8 Sylvia 転送）の Peridot 部分。赤い PP は既存コンセント。A〜C の色枠は電源の扱い（右の凡例）。国名プレートの席割りは配席表（児玉さん 修正案1005）による。準備一覧の「場所」の記号は下の凡例に対応。</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>U 字（28 席）</t>
+          <t>U 字（30 席、底は 3 卓）</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>2 人目の代表、パートナー機関、事務方。電源: 左は左壁から延長タップ、右は追加（見積次第）</t>
+          <t>2 人目の代表、パートナー機関、事務方。電源: 右は右壁から延長タップ、左は追加（見積次第）</t>
         </is>
       </c>
     </row>
@@ -2872,12 +2872,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>シアター席（後方 54 席）</t>
+          <t>シアター席（後方 40 席）</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>一般参加者ほか自由席</t>
+          <t>29 日は SEPDM 40 名。一般参加者の席は不足（Sylvia と調整中）</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>AV 卓（前方左）</t>
+          <t>AV 卓（前方右）</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>ADRC 事務局（AV 卓の隣、前方左 2 卓）</t>
+          <t>ADRC 事務局（AV 卓の隣、前方右 2 卓）</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>三脚、HDMI で AV 卓へ（前方左まで約 20m 以上、延長が必要か業者と確認）。後方壁の既存コンセント</t>
+          <t>三脚、HDMI で AV 卓へ（前方右まで約 20m 以上、延長が必要か業者と確認）。後方壁の既存コンセント</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct camera position to inside the U-shape
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓が EXPO 図面（Peridot 204-206）どおりか。電源: AV 卓・事務局・カメラ位置は既存コンセント＋延長コード、側面列と教室型は見積の結果どおりか。違いがあれば Sylvia と業者に伝える。</t>
+          <t>机・椅子・ステージ・演台・スクリーン・マイク・AV 卓が EXPO 図面（Peridot 204-206）どおりか。電源: AV 卓・事務局は既存コンセント、U 字内のカメラは AV 卓から延長コード、側面列と教室型は見積の結果どおりか。違いがあれば Sylvia と業者に伝える。</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>後方中央。演台・U 字・前方卓が入るか。映像を AV 卓の Zoom 用 PC へ。業者カメラの場合は業者オペと確認し、ADRC のカメラは予備。</t>
+          <t>U 字の内側（中央）。演台・ステージ・U 字の発言者・教室型を振れるか。映像を AV 卓の Zoom 用 PC へ。業者カメラの場合は業者オペと確認し、ADRC のカメラは予備。</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -2940,12 +2940,12 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>カメラ位置（後方中央）</t>
+          <t>カメラ位置（U 字の内側）</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>三脚、HDMI で AV 卓へ（前方右まで約 20m 以上、延長が必要か業者と確認）。後方壁の既存コンセント</t>
+          <t>三脚。HDMI と電源は AV 卓（前方右）から床に這わせてテープ固定。経路で約 12m、手持ちの 10m では足りない見込みで業者と確認</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
U-shape uses 28 of 30 seats
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Giz7vfig8Fz5wHpNCoicZ
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_会場準備一覧_案1008.xlsx
@@ -825,7 +825,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>U 字 30、側面列、教室型の指定席、前方卓（Day1 モデレーター／Day2 TS 登壇者・Co-Chair／SC 用／閉会用）。COSEM が作る参加者名札（パス）とは別。</t>
+          <t>U 字 28、側面列、教室型の指定席、前方卓（Day1 モデレーター／Day2 TS 登壇者・Co-Chair／SC 用／閉会用）。COSEM が作る参加者名札（パス）とは別。</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>U 字 30、側面列、教室型の指定席、前方のモデレーター卓。配席図どおり。</t>
+          <t>U 字 28、側面列、教室型の指定席、前方のモデレーター卓。配席図どおり。</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>U 字（30 席、底は 3 卓）</t>
+          <t>U 字（28 席。図面は 30 席だが両脚の一番下は使わない。底は 3 卓）</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">

</xml_diff>